<commit_message>
Update the RTS check to the 8 Sep dashboard refresh (July 786 t)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PR3GnM6MfmntaD58yeFwca
</commit_message>
<xml_diff>
--- a/Large Market Certificates/RTS_Market_Based_Check_Jul26.xlsx
+++ b/Large Market Certificates/RTS_Market_Based_Check_Jul26.xlsx
@@ -166,7 +166,7 @@
     <t xml:space="preserve">Dashboard less market-based electricity</t>
   </si>
   <si>
-    <t xml:space="preserve">The non-electricity balance the dashboard implies (Scope 1 and anything else). Steady at ~99 t Mar-May and 70 t in Jun; 762 t in Jul</t>
+    <t xml:space="preserve">The non-electricity balance the dashboard implies (Scope 1 and anything else). Steady at ~110 t Mar-May and 86 t in Jun; 620 t in Jul</t>
   </si>
   <si>
     <t xml:space="preserve">Dashboard less location-based electricity</t>
@@ -226,7 +226,7 @@
     <t xml:space="preserve">2. Market-based electricity for RTS FELL in July, from 471.9 t (Jun) to 166.3 t, because those three accounts started crediting on 1 July. The July spike on the dashboard is not coming from the market-based electricity as it stands in the 6 Sep export.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Best fit for the 928 t: the dashboard was refreshed while the old CS Energy accounts at Maryborough (1003077, 1003082) and Torbanlea (1003571) still had no Replaced On and were accruing July (~165 + 7 + 110 = ~282 t) on top of the Engie actuals, and before the certificate accounts were linked. 739 (location-based) + 282 - 171 (HCMT deduction) + ~70-99 non-electricity = 920-950 t. The CS Energy accounts were closed at 30 Jun 26 between the 3 Sep and 5 Sep extracts, so a refresh should clear it. Scope 1 is not in this repo, so I cannot rule out a genuine July scope 1 movement - check gas and fuel for RTS if the refresh does not clear it.</t>
+    <t xml:space="preserve">3. The 8 Sep refresh brought July down from 928 t to 786 t (the CS Energy accounts at Maryborough and Torbanlea closing at 30 Jun removed their July accruals), but July is still ~230 t above June when the electricity says it should be ~300 t below. The gap (~510 t over the Mar-Jun non-electricity run-rate) is close to the two new certificate accounts not being credited at all: Auburn 204.8 t + Maryborough 196.8 t = 401.6 t, plus Torbanlea's high first Engie bill (+56 t). HCMT's deduction IS credited every month and the only structural difference is its factor - LGCs Victoria 25-26 - against the new accounts' 24-25 vintage. If the dashboard's market-based measure only picks up current-year factors, moving the accounts to 25-26 LGC factors fixes both this and item 4. Scope 1 is not in this repo, so a genuine July gas or fuel movement cannot be ruled out.</t>
   </si>
   <si>
     <t xml:space="preserve">4. All three certificate accounts are on 24-25 LGC factors (NSW -0.66, QLD -0.71) against electricity on 25-26 (0.64, 0.67), so each site nets slightly below zero: Auburn -6.2 t, Maryborough -11 t before the foundry issue. Needs the 25-26 LGC factors (already open).</t>
@@ -1421,19 +1421,19 @@
         <v>17</v>
       </c>
       <c r="B9" s="8" t="n">
-        <v>625.05</v>
+        <v>635.78</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>543.82</v>
+        <v>557.14</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>612.33</v>
+        <v>626.46</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>542.12</v>
+        <v>558.22</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>928.48</v>
+        <v>786.33</v>
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="7" t="s">
@@ -1446,23 +1446,23 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">IF(B9="","",B9-B8)</f>
-        <v>98.8004999999999</v>
+        <v>109.5305</v>
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">IF(C9="","",C9-C8)</f>
-        <v>99.0203</v>
+        <v>112.3403</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">IF(D9="","",D9-D8)</f>
-        <v>99.1211000000001</v>
+        <v>113.2511</v>
       </c>
       <c r="E10" s="6" t="n">
         <f aca="false">IF(E9="","",E9-E8)</f>
-        <v>70.2670999999999</v>
+        <v>86.3670999999999</v>
       </c>
       <c r="F10" s="6" t="n">
         <f aca="false">IF(F9="","",F9-F8)</f>
-        <v>762.1732</v>
+        <v>620.0232</v>
       </c>
       <c r="G10" s="6" t="str">
         <f aca="false">IF(G9="","",G9-G8)</f>
@@ -1478,23 +1478,23 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="false">IF(B9="","",B9-B6)</f>
-        <v>-41.9319</v>
+        <v>-31.2019</v>
       </c>
       <c r="C11" s="6" t="n">
         <f aca="false">IF(C9="","",C9-C6)</f>
-        <v>-44.8430999999999</v>
+        <v>-31.5231</v>
       </c>
       <c r="D11" s="6" t="n">
         <f aca="false">IF(D9="","",D9-D6)</f>
-        <v>-60.1383</v>
+        <v>-46.0083</v>
       </c>
       <c r="E11" s="6" t="n">
         <f aca="false">IF(E9="","",E9-E6)</f>
-        <v>-92.4993000000001</v>
+        <v>-76.3993</v>
       </c>
       <c r="F11" s="6" t="n">
         <f aca="false">IF(F9="","",F9-F6)</f>
-        <v>189.4518</v>
+        <v>47.3018</v>
       </c>
       <c r="G11" s="6" t="str">
         <f aca="false">IF(G9="","",G9-G6)</f>

</xml_diff>